<commit_message>
fix: Prawidłowy kod będzie znikał po wpisaniu
</commit_message>
<xml_diff>
--- a/backend/super_safe_file.xlsx
+++ b/backend/super_safe_file.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Eb61mps</t>
+          <t>3PIu7f0</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>BVON7T0</t>
+          <t>Ls6Hdio</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>YvXENJw</t>
+          <t>mCkwEzc</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>xCoq5Qo</t>
+          <t>uWoFKuk</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Sgq1_kU</t>
+          <t>K4Yiegc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: 'sesja', informacja o bledych danych, logout button
</commit_message>
<xml_diff>
--- a/backend/super_safe_file.xlsx
+++ b/backend/super_safe_file.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>3PIu7f0</t>
+          <t>jGSI56M</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Ls6Hdio</t>
+          <t>R_iygpA</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>mCkwEzc</t>
+          <t>FTY2308</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>uWoFKuk</t>
+          <t>LVOrxhY</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>K4Yiegc</t>
+          <t>12HH0pY</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Wyswietlanie plakatow i ocenianie ich
</commit_message>
<xml_diff>
--- a/backend/super_safe_file.xlsx
+++ b/backend/super_safe_file.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>jGSI56M</t>
+          <t>TXv47aI</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>R_iygpA</t>
+          <t>A7Z1h9c</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>FTY2308</t>
+          <t>SzlNWWA</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>LVOrxhY</t>
+          <t>XiFBVC4</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>12HH0pY</t>
+          <t>CnuE2XA</t>
         </is>
       </c>
     </row>

</xml_diff>